<commit_message>
Name the four email-support target companies on Exgrowth's October invoice
The full list overflows the item column, so the line says "4社分" and
the companies are listed in 備考.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GmiXe9RCHpFsdrbpadPUq2
</commit_message>
<xml_diff>
--- a/invoice_agent/exgrowth_202610.xlsx
+++ b/invoice_agent/exgrowth_202610.xlsx
@@ -498,6 +498,11 @@
       <c r="H2" s="1" t="n">
         <v>46326</v>
       </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>メール配信サポート対象：インダストリア様、BNE様、DFT様、日本電力調達ソリューション様</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -510,7 +515,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>メール配信サポート</t>
+          <t>4社分、メール配信サポート（対象は備考参照）</t>
         </is>
       </c>
       <c r="D3" t="n">

</xml_diff>

<commit_message>
Wrap long item names in the invoice table; list Exgrowth's 4 companies inline
Item text that overflowed its column was silently hidden under the next
cell. The item cell now wraps (honoring explicit newlines) and the row
grows to fit. Exgrowth wants target companies listed on each service
line, so the email support line names all four directly instead of
pointing to 備考.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GmiXe9RCHpFsdrbpadPUq2
</commit_message>
<xml_diff>
--- a/invoice_agent/exgrowth_202610.xlsx
+++ b/invoice_agent/exgrowth_202610.xlsx
@@ -498,11 +498,6 @@
       <c r="H2" s="1" t="n">
         <v>46326</v>
       </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>メール配信サポート対象：インダストリア様、BNE様、DFT様、日本電力調達ソリューション様</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -515,7 +510,8 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>4社分、メール配信サポート（対象は備考参照）</t>
+          <t>インダストリア・BNE・DFT・
+日本電力調達ソリューション分、メール配信サポート</t>
         </is>
       </c>
       <c r="D3" t="n">

</xml_diff>

<commit_message>
Date October invoices 10/30 (issued today) instead of month-end
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GmiXe9RCHpFsdrbpadPUq2
</commit_message>
<xml_diff>
--- a/invoice_agent/exgrowth_202610.xlsx
+++ b/invoice_agent/exgrowth_202610.xlsx
@@ -496,7 +496,7 @@
         </is>
       </c>
       <c r="H2" s="1" t="n">
-        <v>46326</v>
+        <v>46325</v>
       </c>
     </row>
     <row r="3">
@@ -506,7 +506,7 @@
         </is>
       </c>
       <c r="B3" s="1" t="n">
-        <v>46326</v>
+        <v>46325</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -529,7 +529,7 @@
         </is>
       </c>
       <c r="H3" s="1" t="n">
-        <v>46326</v>
+        <v>46325</v>
       </c>
     </row>
   </sheetData>

</xml_diff>